<commit_message>
data fixed and more scripts
</commit_message>
<xml_diff>
--- a/data/onboardmeasurements/Peters_Board/Analysis/ImpliedField_Python/Correlation_Summary.xlsx
+++ b/data/onboardmeasurements/Peters_Board/Analysis/ImpliedField_Python/Correlation_Summary.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="75">
   <si>
     <t>Board</t>
   </si>
@@ -35,6 +35,9 @@
   </si>
   <si>
     <t>Correlation_G_per_A</t>
+  </si>
+  <si>
+    <t>RMSE_G</t>
   </si>
   <si>
     <t>Board1</t>
@@ -567,10 +570,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G61"/>
+  <dimension ref="A1:H61"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:8">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -592,16 +595,19 @@
       <c r="G1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:7">
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D2">
         <v>5.647181165083381</v>
@@ -615,16 +621,19 @@
       <c r="G2">
         <v>-1.250150860184813</v>
       </c>
-    </row>
-    <row r="3" spans="1:7">
+      <c r="H2">
+        <v>0.1654120968420386</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D3">
         <v>9.02104485281461</v>
@@ -638,16 +647,19 @@
       <c r="G3">
         <v>-1.188964515632504</v>
       </c>
-    </row>
-    <row r="4" spans="1:7">
+      <c r="H3">
+        <v>0.09705823301767517</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
       <c r="A4" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D4">
         <v>18.05084758996272</v>
@@ -661,16 +673,19 @@
       <c r="G4">
         <v>-1.247759076976988</v>
       </c>
-    </row>
-    <row r="5" spans="1:7">
+      <c r="H4">
+        <v>0.08037554489601152</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
       <c r="A5" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C5" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D5">
         <v>28.07705976307444</v>
@@ -684,16 +699,19 @@
       <c r="G5">
         <v>-1.169432612285825</v>
       </c>
-    </row>
-    <row r="6" spans="1:7">
+      <c r="H5">
+        <v>0.04776929393366686</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
       <c r="A6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C6" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D6">
         <v>52.29807802618812</v>
@@ -707,16 +725,19 @@
       <c r="G6">
         <v>-1.052908646079837</v>
       </c>
-    </row>
-    <row r="7" spans="1:7">
+      <c r="H6">
+        <v>0.02249619384404992</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
       <c r="A7" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C7" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D7">
         <v>3.827045790167987</v>
@@ -730,16 +751,19 @@
       <c r="G7">
         <v>-0.3355301565196502</v>
       </c>
-    </row>
-    <row r="8" spans="1:7">
+      <c r="H7">
+        <v>0.3489467739561518</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
       <c r="A8" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B8" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C8" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D8">
         <v>21.49492102980698</v>
@@ -753,16 +777,19 @@
       <c r="G8">
         <v>-1.156286418740269</v>
       </c>
-    </row>
-    <row r="9" spans="1:7">
+      <c r="H8">
+        <v>0.02468020690300423</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
       <c r="A9" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C9" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D9">
         <v>29.02363877072268</v>
@@ -776,16 +803,19 @@
       <c r="G9">
         <v>-1.213255220593446</v>
       </c>
-    </row>
-    <row r="10" spans="1:7">
+      <c r="H9">
+        <v>0.03630937587840155</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8">
       <c r="A10" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C10" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D10">
         <v>17.01388730630512</v>
@@ -799,16 +829,19 @@
       <c r="G10">
         <v>-1.332886801322913</v>
       </c>
-    </row>
-    <row r="11" spans="1:7">
+      <c r="H10">
+        <v>0.05588565985101152</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8">
       <c r="A11" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B11" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C11" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D11">
         <v>36.5103504343287</v>
@@ -822,16 +855,19 @@
       <c r="G11">
         <v>-1.27054837708283</v>
       </c>
-    </row>
-    <row r="12" spans="1:7">
+      <c r="H11">
+        <v>0.1193814473578211</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8">
       <c r="A12" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B12" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C12" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D12">
         <v>51.58928323396383</v>
@@ -845,16 +881,19 @@
       <c r="G12">
         <v>-1.059693467614076</v>
       </c>
-    </row>
-    <row r="13" spans="1:7">
+      <c r="H12">
+        <v>0.01802079875922517</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8">
       <c r="A13" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B13" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C13" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D13">
         <v>2.931282006370532</v>
@@ -868,16 +907,19 @@
       <c r="G13">
         <v>-1.287014435330869</v>
       </c>
-    </row>
-    <row r="14" spans="1:7">
+      <c r="H13">
+        <v>0.1908985262782041</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8">
       <c r="A14" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B14" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C14" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D14">
         <v>125.2401316686183</v>
@@ -891,16 +933,19 @@
       <c r="G14">
         <v>-1.117046658941634</v>
       </c>
-    </row>
-    <row r="15" spans="1:7">
+      <c r="H14">
+        <v>0.05242003468507922</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8">
       <c r="A15" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B15" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C15" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D15">
         <v>26.7050487191027</v>
@@ -914,16 +959,19 @@
       <c r="G15">
         <v>-1.138527495045671</v>
       </c>
-    </row>
-    <row r="16" spans="1:7">
+      <c r="H15">
+        <v>0.05903971310875113</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8">
       <c r="A16" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B16" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C16" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D16">
         <v>113.0289618455402</v>
@@ -937,16 +985,19 @@
       <c r="G16">
         <v>-0.2712590926949552</v>
       </c>
-    </row>
-    <row r="17" spans="1:7">
+      <c r="H16">
+        <v>0.01353195292532293</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8">
       <c r="A17" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B17" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C17" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D17">
         <v>68.10490981480055</v>
@@ -960,16 +1011,19 @@
       <c r="G17">
         <v>-1.182004614643303</v>
       </c>
-    </row>
-    <row r="18" spans="1:7">
+      <c r="H17">
+        <v>0.03394423913975938</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8">
       <c r="A18" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B18" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C18" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D18">
         <v>83.46815946592136</v>
@@ -983,16 +1037,19 @@
       <c r="G18">
         <v>-1.084484672985766</v>
       </c>
-    </row>
-    <row r="19" spans="1:7">
+      <c r="H18">
+        <v>0.02627866298097563</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8">
       <c r="A19" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B19" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C19" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D19">
         <v>22.17250530772382</v>
@@ -1006,16 +1063,19 @@
       <c r="G19">
         <v>-1.003057578214141</v>
       </c>
-    </row>
-    <row r="20" spans="1:7">
+      <c r="H19">
+        <v>0.2490932135888003</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8">
       <c r="A20" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B20" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C20" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D20">
         <v>12.42723150006206</v>
@@ -1029,16 +1089,19 @@
       <c r="G20">
         <v>-1.24501525964853</v>
       </c>
-    </row>
-    <row r="21" spans="1:7">
+      <c r="H20">
+        <v>0.08062640248238774</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8">
       <c r="A21" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B21" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C21" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D21">
         <v>31.62423391959087</v>
@@ -1052,16 +1115,19 @@
       <c r="G21">
         <v>-1.222901203094112</v>
       </c>
-    </row>
-    <row r="22" spans="1:7">
+      <c r="H21">
+        <v>0.04903073204720567</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8">
       <c r="A22" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B22" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C22" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D22">
         <v>146.4614031390282</v>
@@ -1075,16 +1141,19 @@
       <c r="G22">
         <v>-1.238330216875678</v>
       </c>
-    </row>
-    <row r="23" spans="1:7">
+      <c r="H22">
+        <v>0.0144425677746405</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8">
       <c r="A23" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B23" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C23" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D23">
         <v>97.86566025821391</v>
@@ -1098,16 +1167,19 @@
       <c r="G23">
         <v>-1.191233767905809</v>
       </c>
-    </row>
-    <row r="24" spans="1:7">
+      <c r="H23">
+        <v>0.02341128697454981</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8">
       <c r="A24" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B24" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C24" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D24">
         <v>78.63975910451036</v>
@@ -1121,16 +1193,19 @@
       <c r="G24">
         <v>-1.069395148813229</v>
       </c>
-    </row>
-    <row r="25" spans="1:7">
+      <c r="H24">
+        <v>0.01208880711305554</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8">
       <c r="A25" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B25" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C25" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D25">
         <v>10.24663775290717</v>
@@ -1144,16 +1219,19 @@
       <c r="G25">
         <v>-1.011169617265815</v>
       </c>
-    </row>
-    <row r="26" spans="1:7">
+      <c r="H25">
+        <v>0.1720747126153388</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8">
       <c r="A26" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B26" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C26" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D26">
         <v>73.57743789180142</v>
@@ -1167,16 +1245,19 @@
       <c r="G26">
         <v>-0.9965911174940453</v>
       </c>
-    </row>
-    <row r="27" spans="1:7">
+      <c r="H26">
+        <v>0.05743760351832346</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8">
       <c r="A27" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B27" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C27" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D27">
         <v>50.31676917409693</v>
@@ -1190,16 +1271,19 @@
       <c r="G27">
         <v>-1.102329589037496</v>
       </c>
-    </row>
-    <row r="28" spans="1:7">
+      <c r="H27">
+        <v>0.1089673922558824</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8">
       <c r="A28" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B28" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C28" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D28">
         <v>54.19511506620597</v>
@@ -1213,16 +1297,19 @@
       <c r="G28">
         <v>-1.196415527559085</v>
       </c>
-    </row>
-    <row r="29" spans="1:7">
+      <c r="H28">
+        <v>0.02834230787526099</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8">
       <c r="A29" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B29" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C29" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D29">
         <v>75.34520643297736</v>
@@ -1236,16 +1323,19 @@
       <c r="G29">
         <v>-1.147502677008406</v>
       </c>
-    </row>
-    <row r="30" spans="1:7">
+      <c r="H29">
+        <v>0.03735176102394585</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8">
       <c r="A30" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B30" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C30" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D30">
         <v>85.27318230501869</v>
@@ -1259,16 +1349,19 @@
       <c r="G30">
         <v>-1.111626739139716</v>
       </c>
-    </row>
-    <row r="31" spans="1:7">
+      <c r="H30">
+        <v>0.01326416722233132</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8">
       <c r="A31" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B31" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C31" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D31">
         <v>20.50656116548535</v>
@@ -1282,16 +1375,19 @@
       <c r="G31">
         <v>-0.96703398480209</v>
       </c>
-    </row>
-    <row r="32" spans="1:7">
+      <c r="H31">
+        <v>0.1219832709188648</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8">
       <c r="A32" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B32" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C32" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D32">
         <v>25.14529287861363</v>
@@ -1305,16 +1401,19 @@
       <c r="G32">
         <v>-1.064804708204732</v>
       </c>
-    </row>
-    <row r="33" spans="1:7">
+      <c r="H32">
+        <v>0.04312376780458648</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8">
       <c r="A33" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B33" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C33" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D33">
         <v>37.95945709463887</v>
@@ -1328,16 +1427,19 @@
       <c r="G33">
         <v>-1.06023092334109</v>
       </c>
-    </row>
-    <row r="34" spans="1:7">
+      <c r="H33">
+        <v>0.04013415624161748</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8">
       <c r="A34" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B34" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C34" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D34">
         <v>59.55063119416454</v>
@@ -1351,16 +1453,19 @@
       <c r="G34">
         <v>-1.206224665523016</v>
       </c>
-    </row>
-    <row r="35" spans="1:7">
+      <c r="H34">
+        <v>0.02908355500126322</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8">
       <c r="A35" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B35" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C35" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D35">
         <v>72.57839507479575</v>
@@ -1374,16 +1479,19 @@
       <c r="G35">
         <v>-1.207062351343348</v>
       </c>
-    </row>
-    <row r="36" spans="1:7">
+      <c r="H35">
+        <v>0.02414242681753815</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8">
       <c r="A36" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B36" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C36" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D36">
         <v>95.35641614153549</v>
@@ -1397,16 +1505,19 @@
       <c r="G36">
         <v>-1.109977465555213</v>
       </c>
-    </row>
-    <row r="37" spans="1:7">
+      <c r="H36">
+        <v>0.01192889538873223</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8">
       <c r="A37" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B37" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C37" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D37">
         <v>79.03221943070159</v>
@@ -1420,16 +1531,19 @@
       <c r="G37">
         <v>-1.001349158512698</v>
       </c>
-    </row>
-    <row r="38" spans="1:7">
+      <c r="H37">
+        <v>0.02130834902060431</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8">
       <c r="A38" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B38" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C38" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D38">
         <v>58.62951915213258</v>
@@ -1443,16 +1557,19 @@
       <c r="G38">
         <v>-1.126915043545053</v>
       </c>
-    </row>
-    <row r="39" spans="1:7">
+      <c r="H38">
+        <v>0.05321003216062429</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8">
       <c r="A39" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B39" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C39" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D39">
         <v>72.63890786045005</v>
@@ -1466,16 +1583,19 @@
       <c r="G39">
         <v>-1.175470651749928</v>
       </c>
-    </row>
-    <row r="40" spans="1:7">
+      <c r="H39">
+        <v>0.0489767771866955</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8">
       <c r="A40" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B40" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C40" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D40">
         <v>83.05777431098903</v>
@@ -1489,16 +1609,19 @@
       <c r="G40">
         <v>-1.237258970503794</v>
       </c>
-    </row>
-    <row r="41" spans="1:7">
+      <c r="H40">
+        <v>0.04978529067558385</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8">
       <c r="A41" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B41" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C41" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D41">
         <v>99.27568574445569</v>
@@ -1512,16 +1635,19 @@
       <c r="G41">
         <v>-1.15964041747908</v>
       </c>
-    </row>
-    <row r="42" spans="1:7">
+      <c r="H41">
+        <v>0.01807839158434938</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8">
       <c r="A42" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B42" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C42" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D42">
         <v>88.37552930160459</v>
@@ -1535,16 +1661,19 @@
       <c r="G42">
         <v>-1.03164739968384</v>
       </c>
-    </row>
-    <row r="43" spans="1:7">
+      <c r="H42">
+        <v>0.009432038055530008</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8">
       <c r="A43" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B43" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C43" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D43">
         <v>47.35222453074022</v>
@@ -1558,16 +1687,19 @@
       <c r="G43">
         <v>-0.9249986793065145</v>
       </c>
-    </row>
-    <row r="44" spans="1:7">
+      <c r="H43">
+        <v>0.08443146555095914</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8">
       <c r="A44" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B44" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C44" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D44">
         <v>49.57694218410126</v>
@@ -1581,16 +1713,19 @@
       <c r="G44">
         <v>-1.034590858054074</v>
       </c>
-    </row>
-    <row r="45" spans="1:7">
+      <c r="H44">
+        <v>0.06277177630658007</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8">
       <c r="A45" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B45" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C45" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D45">
         <v>76.63808537263186</v>
@@ -1604,16 +1739,19 @@
       <c r="G45">
         <v>-1.248538759133305</v>
       </c>
-    </row>
-    <row r="46" spans="1:7">
+      <c r="H45">
+        <v>0.03098870296615478</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8">
       <c r="A46" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B46" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C46" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D46">
         <v>84.75048372380536</v>
@@ -1627,16 +1765,19 @@
       <c r="G46">
         <v>-1.183416319241447</v>
       </c>
-    </row>
-    <row r="47" spans="1:7">
+      <c r="H46">
+        <v>0.04844182101246117</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8">
       <c r="A47" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B47" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C47" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D47">
         <v>83.13428807361933</v>
@@ -1650,16 +1791,19 @@
       <c r="G47">
         <v>-1.139248099852525</v>
       </c>
-    </row>
-    <row r="48" spans="1:7">
+      <c r="H47">
+        <v>0.01889493132586367</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8">
       <c r="A48" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B48" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C48" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D48">
         <v>2269.207651915169</v>
@@ -1673,16 +1817,19 @@
       <c r="G48">
         <v>-121.5676802966202</v>
       </c>
-    </row>
-    <row r="49" spans="1:7">
+      <c r="H48">
+        <v>255.2353512560123</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8">
       <c r="A49" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B49" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C49" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D49">
         <v>51.78490498697956</v>
@@ -1696,16 +1843,19 @@
       <c r="G49">
         <v>-0.851967352077575</v>
       </c>
-    </row>
-    <row r="50" spans="1:7">
+      <c r="H49">
+        <v>0.1729359348681366</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8">
       <c r="A50" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B50" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C50" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D50">
         <v>7.414270876933209</v>
@@ -1719,16 +1869,19 @@
       <c r="G50">
         <v>-1.141313005996113</v>
       </c>
-    </row>
-    <row r="51" spans="1:7">
+      <c r="H50">
+        <v>0.1672137576914152</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8">
       <c r="A51" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B51" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C51" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D51">
         <v>13.48998729811724</v>
@@ -1742,16 +1895,19 @@
       <c r="G51">
         <v>-1.128853922064218</v>
       </c>
-    </row>
-    <row r="52" spans="1:7">
+      <c r="H51">
+        <v>0.06368918367593454</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8">
       <c r="A52" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B52" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C52" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D52">
         <v>24.90324173599608</v>
@@ -1765,16 +1921,19 @@
       <c r="G52">
         <v>-1.160141780253347</v>
       </c>
-    </row>
-    <row r="53" spans="1:7">
+      <c r="H52">
+        <v>0.04290000302312324</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8">
       <c r="A53" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B53" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C53" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D53">
         <v>35.8133866675048</v>
@@ -1788,16 +1947,19 @@
       <c r="G53">
         <v>-1.136076565694146</v>
       </c>
-    </row>
-    <row r="54" spans="1:7">
+      <c r="H53">
+        <v>0.03206734117157507</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8">
       <c r="A54" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B54" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C54" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D54">
         <v>62.92001142089412</v>
@@ -1811,16 +1973,19 @@
       <c r="G54">
         <v>-1.071566303122123</v>
       </c>
-    </row>
-    <row r="55" spans="1:7">
+      <c r="H54">
+        <v>0.01359098568294228</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8">
       <c r="A55" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B55" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C55" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D55">
         <v>74.75504147874878</v>
@@ -1834,16 +1999,19 @@
       <c r="G55">
         <v>-0.9741691125068884</v>
       </c>
-    </row>
-    <row r="56" spans="1:7">
+      <c r="H55">
+        <v>0.04179688413380851</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8">
       <c r="A56" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B56" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C56" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D56">
         <v>6.356654786633988</v>
@@ -1857,16 +2025,19 @@
       <c r="G56">
         <v>-1.047383335141998</v>
       </c>
-    </row>
-    <row r="57" spans="1:7">
+      <c r="H56">
+        <v>0.1358014739224134</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8">
       <c r="A57" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B57" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C57" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D57">
         <v>12.33646232158047</v>
@@ -1880,16 +2051,19 @@
       <c r="G57">
         <v>-1.157916392185165</v>
       </c>
-    </row>
-    <row r="58" spans="1:7">
+      <c r="H57">
+        <v>0.06890293652652933</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8">
       <c r="A58" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B58" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C58" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D58">
         <v>21.98922138963593</v>
@@ -1903,16 +2077,19 @@
       <c r="G58">
         <v>-1.247782417751954</v>
       </c>
-    </row>
-    <row r="59" spans="1:7">
+      <c r="H58">
+        <v>0.04550107762404755</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8">
       <c r="A59" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B59" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C59" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D59">
         <v>36.09762220396794</v>
@@ -1926,16 +2103,19 @@
       <c r="G59">
         <v>-1.179786253518166</v>
       </c>
-    </row>
-    <row r="60" spans="1:7">
+      <c r="H59">
+        <v>0.03241921170643407</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8">
       <c r="A60" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B60" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C60" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D60">
         <v>58.31599697902271</v>
@@ -1949,16 +2129,19 @@
       <c r="G60">
         <v>-1.109437764121858</v>
       </c>
-    </row>
-    <row r="61" spans="1:7">
+      <c r="H60">
+        <v>0.02200307295368992</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8">
       <c r="A61" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B61" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C61" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D61">
         <v>61.46130417439842</v>
@@ -1971,6 +2154,9 @@
       </c>
       <c r="G61">
         <v>-0.9979109712542467</v>
+      </c>
+      <c r="H61">
+        <v>0.04366557286781613</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fixes for the plot
</commit_message>
<xml_diff>
--- a/data/onboardmeasurements/Peters_Board/Analysis/ImpliedField_Python/Correlation_Summary.xlsx
+++ b/data/onboardmeasurements/Peters_Board/Analysis/ImpliedField_Python/Correlation_Summary.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="75">
   <si>
     <t>Board</t>
   </si>
@@ -570,7 +570,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H61"/>
+  <dimension ref="A1:H63"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -613,7 +613,7 @@
         <v>5.647181165083381</v>
       </c>
       <c r="E2">
-        <v>1.880584257800381</v>
+        <v>1.214765349200426</v>
       </c>
       <c r="F2">
         <v>0.49963</v>
@@ -639,7 +639,7 @@
         <v>9.02104485281461</v>
       </c>
       <c r="E3">
-        <v>1.427772526369687</v>
+        <v>0.621879182681398</v>
       </c>
       <c r="F3">
         <v>0.49963</v>
@@ -665,13 +665,13 @@
         <v>18.05084758996272</v>
       </c>
       <c r="E4">
-        <v>1.311295765034733</v>
+        <v>0.8730891954771963</v>
       </c>
       <c r="F4">
         <v>0.49963</v>
       </c>
       <c r="G4">
-        <v>-1.247759076976988</v>
+        <v>-1.247759076976987</v>
       </c>
       <c r="H4">
         <v>0.08037554489601152</v>
@@ -691,7 +691,7 @@
         <v>28.07705976307444</v>
       </c>
       <c r="E5">
-        <v>1.190651737827825</v>
+        <v>0.6499968356373802</v>
       </c>
       <c r="F5">
         <v>0.49963</v>
@@ -717,16 +717,16 @@
         <v>52.29807802618812</v>
       </c>
       <c r="E6">
-        <v>1.096981039556893</v>
+        <v>0.5445706816555408</v>
       </c>
       <c r="F6">
         <v>0.49963</v>
       </c>
       <c r="G6">
-        <v>-1.052908646079837</v>
+        <v>-1.052908646079836</v>
       </c>
       <c r="H6">
-        <v>0.02249619384404992</v>
+        <v>0.02249619384404993</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -743,13 +743,13 @@
         <v>3.827045790167987</v>
       </c>
       <c r="E7">
-        <v>2.610368557823483</v>
+        <v>1.03735367112681</v>
       </c>
       <c r="F7">
         <v>0.49963</v>
       </c>
       <c r="G7">
-        <v>-0.3355301565196502</v>
+        <v>-0.3355301565196496</v>
       </c>
       <c r="H7">
         <v>0.3489467739561518</v>
@@ -769,7 +769,7 @@
         <v>21.49492102980698</v>
       </c>
       <c r="E8">
-        <v>1.182139723368487</v>
+        <v>0.5866502129742328</v>
       </c>
       <c r="F8">
         <v>0.49963</v>
@@ -778,7 +778,7 @@
         <v>-1.156286418740269</v>
       </c>
       <c r="H8">
-        <v>0.02468020690300423</v>
+        <v>0.02468020690300422</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -795,7 +795,7 @@
         <v>29.02363877072268</v>
       </c>
       <c r="E9">
-        <v>1.231065487075943</v>
+        <v>0.5950322127567874</v>
       </c>
       <c r="F9">
         <v>0.49963</v>
@@ -821,13 +821,13 @@
         <v>17.01388730630512</v>
       </c>
       <c r="E10">
-        <v>1.435298092690936</v>
+        <v>0.684734757569725</v>
       </c>
       <c r="F10">
         <v>0.49963</v>
       </c>
       <c r="G10">
-        <v>-1.332886801322913</v>
+        <v>-1.332886801322912</v>
       </c>
       <c r="H10">
         <v>0.05588565985101152</v>
@@ -847,7 +847,7 @@
         <v>36.5103504343287</v>
       </c>
       <c r="E11">
-        <v>1.55599711654869</v>
+        <v>1.10680942580055</v>
       </c>
       <c r="F11">
         <v>0.49963</v>
@@ -873,7 +873,7 @@
         <v>51.58928323396383</v>
       </c>
       <c r="E12">
-        <v>1.083946054191024</v>
+        <v>0.5702734784388239</v>
       </c>
       <c r="F12">
         <v>0.49963</v>
@@ -899,13 +899,13 @@
         <v>2.931282006370532</v>
       </c>
       <c r="E13">
-        <v>1.975244956783495</v>
+        <v>1.497638231483244</v>
       </c>
       <c r="F13">
         <v>0.49963</v>
       </c>
       <c r="G13">
-        <v>-1.287014435330869</v>
+        <v>-1.287014435330868</v>
       </c>
       <c r="H13">
         <v>0.1908985262782041</v>
@@ -925,16 +925,16 @@
         <v>125.2401316686183</v>
       </c>
       <c r="E14">
-        <v>1.176140571216739</v>
+        <v>0.60922963736477</v>
       </c>
       <c r="F14">
         <v>0.49998</v>
       </c>
       <c r="G14">
-        <v>-1.117046658941634</v>
+        <v>-1.117046658941633</v>
       </c>
       <c r="H14">
-        <v>0.05242003468507922</v>
+        <v>0.05242003468507923</v>
       </c>
     </row>
     <row r="15" spans="1:8">
@@ -951,7 +951,7 @@
         <v>26.7050487191027</v>
       </c>
       <c r="E15">
-        <v>1.314732669814814</v>
+        <v>0.7249565504874722</v>
       </c>
       <c r="F15">
         <v>0.49963</v>
@@ -977,13 +977,13 @@
         <v>113.0289618455402</v>
       </c>
       <c r="E16">
-        <v>0.2955879577630726</v>
+        <v>0.1640287559690827</v>
       </c>
       <c r="F16">
         <v>0.49963</v>
       </c>
       <c r="G16">
-        <v>-0.2712590926949552</v>
+        <v>-0.2712590926949551</v>
       </c>
       <c r="H16">
         <v>0.01353195292532293</v>
@@ -1003,7 +1003,7 @@
         <v>68.10490981480055</v>
       </c>
       <c r="E17">
-        <v>1.224581314721556</v>
+        <v>0.6072983594350525</v>
       </c>
       <c r="F17">
         <v>0.49963</v>
@@ -1012,7 +1012,7 @@
         <v>-1.182004614643303</v>
       </c>
       <c r="H17">
-        <v>0.03394423913975938</v>
+        <v>0.03394423913975937</v>
       </c>
     </row>
     <row r="18" spans="1:8">
@@ -1029,7 +1029,7 @@
         <v>83.46815946592136</v>
       </c>
       <c r="E18">
-        <v>1.147263826262899</v>
+        <v>0.5747101686073059</v>
       </c>
       <c r="F18">
         <v>0.49963</v>
@@ -1038,7 +1038,7 @@
         <v>-1.084484672985766</v>
       </c>
       <c r="H18">
-        <v>0.02627866298097563</v>
+        <v>0.02627866298097564</v>
       </c>
     </row>
     <row r="19" spans="1:8">
@@ -1055,7 +1055,7 @@
         <v>22.17250530772382</v>
       </c>
       <c r="E19">
-        <v>2.835042730967493</v>
+        <v>0.7076331601795443</v>
       </c>
       <c r="F19">
         <v>0.49963</v>
@@ -1081,7 +1081,7 @@
         <v>12.42723150006206</v>
       </c>
       <c r="E20">
-        <v>1.667306189628615</v>
+        <v>0.941480811711437</v>
       </c>
       <c r="F20">
         <v>0.49963</v>
@@ -1107,7 +1107,7 @@
         <v>31.62423391959087</v>
       </c>
       <c r="E21">
-        <v>1.280347220519225</v>
+        <v>0.7155904569115377</v>
       </c>
       <c r="F21">
         <v>0.49963</v>
@@ -1133,7 +1133,7 @@
         <v>146.4614031390282</v>
       </c>
       <c r="E22">
-        <v>1.24749590051769</v>
+        <v>0.6239869210678505</v>
       </c>
       <c r="F22">
         <v>0.49963</v>
@@ -1159,13 +1159,13 @@
         <v>97.86566025821391</v>
       </c>
       <c r="E23">
-        <v>1.220039794193157</v>
+        <v>0.6549794875023681</v>
       </c>
       <c r="F23">
         <v>0.49963</v>
       </c>
       <c r="G23">
-        <v>-1.191233767905809</v>
+        <v>-1.19123376790581</v>
       </c>
       <c r="H23">
         <v>0.02341128697454981</v>
@@ -1185,7 +1185,7 @@
         <v>78.63975910451036</v>
       </c>
       <c r="E24">
-        <v>1.077571968237854</v>
+        <v>0.5434909832721833</v>
       </c>
       <c r="F24">
         <v>0.49963</v>
@@ -1211,13 +1211,13 @@
         <v>10.24663775290717</v>
       </c>
       <c r="E25">
-        <v>1.3741092775537</v>
+        <v>0.5816542112370625</v>
       </c>
       <c r="F25">
         <v>0.49963</v>
       </c>
       <c r="G25">
-        <v>-1.011169617265815</v>
+        <v>-1.011169617265814</v>
       </c>
       <c r="H25">
         <v>0.1720747126153388</v>
@@ -1237,7 +1237,7 @@
         <v>73.57743789180142</v>
       </c>
       <c r="E26">
-        <v>1.107948337639624</v>
+        <v>0.6129596421436579</v>
       </c>
       <c r="F26">
         <v>0.49963</v>
@@ -1263,7 +1263,7 @@
         <v>50.31676917409693</v>
       </c>
       <c r="E27">
-        <v>1.646170876222367</v>
+        <v>0.5689951972262833</v>
       </c>
       <c r="F27">
         <v>0.49963</v>
@@ -1289,7 +1289,7 @@
         <v>54.19511506620597</v>
       </c>
       <c r="E28">
-        <v>1.250297188542134</v>
+        <v>0.5911971948182565</v>
       </c>
       <c r="F28">
         <v>0.49963</v>
@@ -1315,7 +1315,7 @@
         <v>75.34520643297736</v>
       </c>
       <c r="E29">
-        <v>1.281966094099394</v>
+        <v>0.6245918251197502</v>
       </c>
       <c r="F29">
         <v>0.49963</v>
@@ -1324,7 +1324,7 @@
         <v>-1.147502677008406</v>
       </c>
       <c r="H29">
-        <v>0.03735176102394585</v>
+        <v>0.03735176102394584</v>
       </c>
     </row>
     <row r="30" spans="1:8">
@@ -1341,7 +1341,7 @@
         <v>85.27318230501869</v>
       </c>
       <c r="E30">
-        <v>1.12086821924994</v>
+        <v>0.5728647469173144</v>
       </c>
       <c r="F30">
         <v>0.49963</v>
@@ -1350,7 +1350,7 @@
         <v>-1.111626739139716</v>
       </c>
       <c r="H30">
-        <v>0.01326416722233132</v>
+        <v>0.01326416722233131</v>
       </c>
     </row>
     <row r="31" spans="1:8">
@@ -1367,13 +1367,13 @@
         <v>20.50656116548535</v>
       </c>
       <c r="E31">
-        <v>1.123542841438809</v>
+        <v>0.6612517764721613</v>
       </c>
       <c r="F31">
         <v>0.49963</v>
       </c>
       <c r="G31">
-        <v>-0.96703398480209</v>
+        <v>-0.9670339848020897</v>
       </c>
       <c r="H31">
         <v>0.1219832709188648</v>
@@ -1393,7 +1393,7 @@
         <v>25.14529287861363</v>
       </c>
       <c r="E32">
-        <v>1.162046516660505</v>
+        <v>0.5472197148956288</v>
       </c>
       <c r="F32">
         <v>0.49963</v>
@@ -1419,7 +1419,7 @@
         <v>37.95945709463887</v>
       </c>
       <c r="E33">
-        <v>1.158341118798856</v>
+        <v>0.4631256963494513</v>
       </c>
       <c r="F33">
         <v>0.49963</v>
@@ -1445,13 +1445,13 @@
         <v>59.55063119416454</v>
       </c>
       <c r="E34">
-        <v>1.278743792852631</v>
+        <v>0.6322351122901878</v>
       </c>
       <c r="F34">
         <v>0.49963</v>
       </c>
       <c r="G34">
-        <v>-1.206224665523016</v>
+        <v>-1.206224665523017</v>
       </c>
       <c r="H34">
         <v>0.02908355500126322</v>
@@ -1471,7 +1471,7 @@
         <v>72.57839507479575</v>
       </c>
       <c r="E35">
-        <v>1.254505557833998</v>
+        <v>0.6234637725643776</v>
       </c>
       <c r="F35">
         <v>0.49963</v>
@@ -1497,7 +1497,7 @@
         <v>95.35641614153549</v>
       </c>
       <c r="E36">
-        <v>1.133641598270095</v>
+        <v>0.5562289581151492</v>
       </c>
       <c r="F36">
         <v>0.49963</v>
@@ -1506,7 +1506,7 @@
         <v>-1.109977465555213</v>
       </c>
       <c r="H36">
-        <v>0.01192889538873223</v>
+        <v>0.01192889538873222</v>
       </c>
     </row>
     <row r="37" spans="1:8">
@@ -1523,13 +1523,13 @@
         <v>79.03221943070159</v>
       </c>
       <c r="E37">
-        <v>1.036792343556167</v>
+        <v>0.5300369937950451</v>
       </c>
       <c r="F37">
         <v>0.49963</v>
       </c>
       <c r="G37">
-        <v>-1.001349158512698</v>
+        <v>-1.001349158512697</v>
       </c>
       <c r="H37">
         <v>0.02130834902060431</v>
@@ -1549,13 +1549,13 @@
         <v>58.62951915213258</v>
       </c>
       <c r="E38">
-        <v>1.162895431959432</v>
+        <v>0.597821720301931</v>
       </c>
       <c r="F38">
         <v>0.49963</v>
       </c>
       <c r="G38">
-        <v>-1.126915043545053</v>
+        <v>-1.126915043545052</v>
       </c>
       <c r="H38">
         <v>0.05321003216062429</v>
@@ -1575,7 +1575,7 @@
         <v>72.63890786045005</v>
       </c>
       <c r="E39">
-        <v>1.242171759704055</v>
+        <v>0.717246466591747</v>
       </c>
       <c r="F39">
         <v>0.49963</v>
@@ -1584,7 +1584,7 @@
         <v>-1.175470651749928</v>
       </c>
       <c r="H39">
-        <v>0.0489767771866955</v>
+        <v>0.04897677718669551</v>
       </c>
     </row>
     <row r="40" spans="1:8">
@@ -1601,13 +1601,13 @@
         <v>83.05777431098903</v>
       </c>
       <c r="E40">
-        <v>1.294520601977876</v>
+        <v>0.635340886964055</v>
       </c>
       <c r="F40">
         <v>0.49963</v>
       </c>
       <c r="G40">
-        <v>-1.237258970503794</v>
+        <v>-1.237258970503793</v>
       </c>
       <c r="H40">
         <v>0.04978529067558385</v>
@@ -1627,13 +1627,13 @@
         <v>99.27568574445569</v>
       </c>
       <c r="E41">
-        <v>1.176219525701044</v>
+        <v>0.5722448510326243</v>
       </c>
       <c r="F41">
         <v>0.49963</v>
       </c>
       <c r="G41">
-        <v>-1.15964041747908</v>
+        <v>-1.159640417479079</v>
       </c>
       <c r="H41">
         <v>0.01807839158434938</v>
@@ -1653,7 +1653,7 @@
         <v>88.37552930160459</v>
       </c>
       <c r="E42">
-        <v>1.048140822827474</v>
+        <v>0.5136037131398012</v>
       </c>
       <c r="F42">
         <v>0.49963</v>
@@ -1662,7 +1662,7 @@
         <v>-1.03164739968384</v>
       </c>
       <c r="H42">
-        <v>0.009432038055530008</v>
+        <v>0.00943203805553001</v>
       </c>
     </row>
     <row r="43" spans="1:8">
@@ -1679,13 +1679,13 @@
         <v>47.35222453074022</v>
       </c>
       <c r="E43">
-        <v>1.074923100327648</v>
+        <v>0.449820472239384</v>
       </c>
       <c r="F43">
         <v>0.49963</v>
       </c>
       <c r="G43">
-        <v>-0.9249986793065145</v>
+        <v>-0.9249986793065148</v>
       </c>
       <c r="H43">
         <v>0.08443146555095914</v>
@@ -1705,13 +1705,13 @@
         <v>49.57694218410126</v>
       </c>
       <c r="E44">
-        <v>1.274181044999103</v>
+        <v>0.6821719636197755</v>
       </c>
       <c r="F44">
         <v>0.49963</v>
       </c>
       <c r="G44">
-        <v>-1.034590858054074</v>
+        <v>-1.034590858054075</v>
       </c>
       <c r="H44">
         <v>0.06277177630658007</v>
@@ -1731,7 +1731,7 @@
         <v>76.63808537263186</v>
       </c>
       <c r="E45">
-        <v>1.292960275797579</v>
+        <v>0.7113956427134216</v>
       </c>
       <c r="F45">
         <v>0.49963</v>
@@ -1740,7 +1740,7 @@
         <v>-1.248538759133305</v>
       </c>
       <c r="H45">
-        <v>0.03098870296615478</v>
+        <v>0.03098870296615477</v>
       </c>
     </row>
     <row r="46" spans="1:8">
@@ -1757,7 +1757,7 @@
         <v>84.75048372380536</v>
       </c>
       <c r="E46">
-        <v>1.295095852876702</v>
+        <v>0.7471343786822681</v>
       </c>
       <c r="F46">
         <v>0.49963</v>
@@ -1766,7 +1766,7 @@
         <v>-1.183416319241447</v>
       </c>
       <c r="H46">
-        <v>0.04844182101246117</v>
+        <v>0.04844182101246118</v>
       </c>
     </row>
     <row r="47" spans="1:8">
@@ -1783,16 +1783,16 @@
         <v>83.13428807361933</v>
       </c>
       <c r="E47">
-        <v>1.161734853788314</v>
+        <v>0.602639430262997</v>
       </c>
       <c r="F47">
         <v>0.49963</v>
       </c>
       <c r="G47">
-        <v>-1.139248099852525</v>
+        <v>-1.139248099852526</v>
       </c>
       <c r="H47">
-        <v>0.01889493132586367</v>
+        <v>0.01889493132586368</v>
       </c>
     </row>
     <row r="48" spans="1:8">
@@ -1809,13 +1809,13 @@
         <v>2269.207651915169</v>
       </c>
       <c r="E48">
-        <v>3675.560494854088</v>
+        <v>3636.176703809415</v>
       </c>
       <c r="F48">
         <v>0.49963</v>
       </c>
       <c r="G48">
-        <v>-121.5676802966202</v>
+        <v>-121.5676802966204</v>
       </c>
       <c r="H48">
         <v>255.2353512560123</v>
@@ -1835,13 +1835,13 @@
         <v>51.78490498697956</v>
       </c>
       <c r="E49">
-        <v>1.347883133464336</v>
+        <v>0.8882897441168603</v>
       </c>
       <c r="F49">
         <v>0.49963</v>
       </c>
       <c r="G49">
-        <v>-0.851967352077575</v>
+        <v>-0.8519673520775748</v>
       </c>
       <c r="H49">
         <v>0.1729359348681366</v>
@@ -1849,54 +1849,54 @@
     </row>
     <row r="50" spans="1:8">
       <c r="A50" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B50" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C50" t="s">
-        <v>63</v>
+        <v>51</v>
       </c>
       <c r="D50">
-        <v>7.414270876933209</v>
+        <v>58.62951915213258</v>
       </c>
       <c r="E50">
-        <v>1.634685352231946</v>
+        <v>0.597821720301931</v>
       </c>
       <c r="F50">
         <v>0.49963</v>
       </c>
       <c r="G50">
-        <v>-1.141313005996113</v>
+        <v>-1.126915043545052</v>
       </c>
       <c r="H50">
-        <v>0.1672137576914152</v>
+        <v>0.05321003216062429</v>
       </c>
     </row>
     <row r="51" spans="1:8">
       <c r="A51" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B51" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C51" t="s">
-        <v>64</v>
+        <v>52</v>
       </c>
       <c r="D51">
-        <v>13.48998729811724</v>
+        <v>72.63890786045005</v>
       </c>
       <c r="E51">
-        <v>1.218681651560696</v>
+        <v>0.717246466591747</v>
       </c>
       <c r="F51">
         <v>0.49963</v>
       </c>
       <c r="G51">
-        <v>-1.128853922064218</v>
+        <v>-1.175470651749928</v>
       </c>
       <c r="H51">
-        <v>0.06368918367593454</v>
+        <v>0.04897677718669551</v>
       </c>
     </row>
     <row r="52" spans="1:8">
@@ -1907,22 +1907,22 @@
         <v>14</v>
       </c>
       <c r="C52" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D52">
-        <v>24.90324173599608</v>
+        <v>7.414270876933209</v>
       </c>
       <c r="E52">
-        <v>1.260880022483476</v>
+        <v>0.980541461281381</v>
       </c>
       <c r="F52">
         <v>0.49963</v>
       </c>
       <c r="G52">
-        <v>-1.160141780253347</v>
+        <v>-1.141313005996112</v>
       </c>
       <c r="H52">
-        <v>0.04290000302312324</v>
+        <v>0.1672137576914152</v>
       </c>
     </row>
     <row r="53" spans="1:8">
@@ -1933,22 +1933,22 @@
         <v>14</v>
       </c>
       <c r="C53" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D53">
-        <v>35.8133866675048</v>
+        <v>13.48998729811724</v>
       </c>
       <c r="E53">
-        <v>1.197317651025293</v>
+        <v>0.6226840555419811</v>
       </c>
       <c r="F53">
         <v>0.49963</v>
       </c>
       <c r="G53">
-        <v>-1.136076565694146</v>
+        <v>-1.128853922064218</v>
       </c>
       <c r="H53">
-        <v>0.03206734117157507</v>
+        <v>0.06368918367593454</v>
       </c>
     </row>
     <row r="54" spans="1:8">
@@ -1959,22 +1959,22 @@
         <v>14</v>
       </c>
       <c r="C54" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D54">
-        <v>62.92001142089412</v>
+        <v>24.90324173599608</v>
       </c>
       <c r="E54">
-        <v>1.079783656514741</v>
+        <v>0.6083545331407918</v>
       </c>
       <c r="F54">
         <v>0.49963</v>
       </c>
       <c r="G54">
-        <v>-1.071566303122123</v>
+        <v>-1.160141780253348</v>
       </c>
       <c r="H54">
-        <v>0.01359098568294228</v>
+        <v>0.04290000302312325</v>
       </c>
     </row>
     <row r="55" spans="1:8">
@@ -1985,22 +1985,22 @@
         <v>14</v>
       </c>
       <c r="C55" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D55">
-        <v>74.75504147874878</v>
+        <v>35.8133866675048</v>
       </c>
       <c r="E55">
-        <v>1.068958004962383</v>
+        <v>0.6279774713516333</v>
       </c>
       <c r="F55">
         <v>0.49963</v>
       </c>
       <c r="G55">
-        <v>-0.9741691125068884</v>
+        <v>-1.136076565694146</v>
       </c>
       <c r="H55">
-        <v>0.04179688413380851</v>
+        <v>0.03206734117157508</v>
       </c>
     </row>
     <row r="56" spans="1:8">
@@ -2011,22 +2011,22 @@
         <v>14</v>
       </c>
       <c r="C56" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D56">
-        <v>6.356654786633988</v>
+        <v>62.92001142089412</v>
       </c>
       <c r="E56">
-        <v>1.507081998559706</v>
+        <v>0.4918943798811738</v>
       </c>
       <c r="F56">
         <v>0.49963</v>
       </c>
       <c r="G56">
-        <v>-1.047383335141998</v>
+        <v>-1.071566303122122</v>
       </c>
       <c r="H56">
-        <v>0.1358014739224134</v>
+        <v>0.01359098568294228</v>
       </c>
     </row>
     <row r="57" spans="1:8">
@@ -2037,22 +2037,22 @@
         <v>14</v>
       </c>
       <c r="C57" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D57">
-        <v>12.33646232158047</v>
+        <v>74.75504147874878</v>
       </c>
       <c r="E57">
-        <v>1.308316726405862</v>
+        <v>0.5246468896836951</v>
       </c>
       <c r="F57">
         <v>0.49963</v>
       </c>
       <c r="G57">
-        <v>-1.157916392185165</v>
+        <v>-0.9741691125068891</v>
       </c>
       <c r="H57">
-        <v>0.06890293652652933</v>
+        <v>0.04179688413380851</v>
       </c>
     </row>
     <row r="58" spans="1:8">
@@ -2063,22 +2063,22 @@
         <v>14</v>
       </c>
       <c r="C58" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D58">
-        <v>21.98922138963593</v>
+        <v>6.356654786633988</v>
       </c>
       <c r="E58">
-        <v>1.303365839661411</v>
+        <v>0.9533316191308537</v>
       </c>
       <c r="F58">
         <v>0.49963</v>
       </c>
       <c r="G58">
-        <v>-1.247782417751954</v>
+        <v>-1.047383335141998</v>
       </c>
       <c r="H58">
-        <v>0.04550107762404755</v>
+        <v>0.1358014739224134</v>
       </c>
     </row>
     <row r="59" spans="1:8">
@@ -2089,22 +2089,22 @@
         <v>14</v>
       </c>
       <c r="C59" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="D59">
-        <v>36.09762220396794</v>
+        <v>12.33646232158047</v>
       </c>
       <c r="E59">
-        <v>1.192045275360793</v>
+        <v>0.7319764584537694</v>
       </c>
       <c r="F59">
         <v>0.49963</v>
       </c>
       <c r="G59">
-        <v>-1.179786253518166</v>
+        <v>-1.157916392185165</v>
       </c>
       <c r="H59">
-        <v>0.03241921170643407</v>
+        <v>0.06890293652652933</v>
       </c>
     </row>
     <row r="60" spans="1:8">
@@ -2115,22 +2115,22 @@
         <v>14</v>
       </c>
       <c r="C60" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D60">
-        <v>58.31599697902271</v>
+        <v>21.98922138963593</v>
       </c>
       <c r="E60">
-        <v>1.124219826398248</v>
+        <v>0.6330374210775421</v>
       </c>
       <c r="F60">
         <v>0.49963</v>
       </c>
       <c r="G60">
-        <v>-1.109437764121858</v>
+        <v>-1.247782417751954</v>
       </c>
       <c r="H60">
-        <v>0.02200307295368992</v>
+        <v>0.04550107762404755</v>
       </c>
     </row>
     <row r="61" spans="1:8">
@@ -2141,22 +2141,74 @@
         <v>14</v>
       </c>
       <c r="C61" t="s">
+        <v>72</v>
+      </c>
+      <c r="D61">
+        <v>36.09762220396794</v>
+      </c>
+      <c r="E61">
+        <v>0.6817623571143527</v>
+      </c>
+      <c r="F61">
+        <v>0.49963</v>
+      </c>
+      <c r="G61">
+        <v>-1.179786253518166</v>
+      </c>
+      <c r="H61">
+        <v>0.03241921170643407</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8">
+      <c r="A62" t="s">
+        <v>12</v>
+      </c>
+      <c r="B62" t="s">
+        <v>14</v>
+      </c>
+      <c r="C62" t="s">
+        <v>73</v>
+      </c>
+      <c r="D62">
+        <v>58.31599697902271</v>
+      </c>
+      <c r="E62">
+        <v>0.5535359364877277</v>
+      </c>
+      <c r="F62">
+        <v>0.49963</v>
+      </c>
+      <c r="G62">
+        <v>-1.109437764121859</v>
+      </c>
+      <c r="H62">
+        <v>0.02200307295368992</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8">
+      <c r="A63" t="s">
+        <v>12</v>
+      </c>
+      <c r="B63" t="s">
+        <v>14</v>
+      </c>
+      <c r="C63" t="s">
         <v>74</v>
       </c>
-      <c r="D61">
+      <c r="D63">
         <v>61.46130417439842</v>
       </c>
-      <c r="E61">
-        <v>1.097438476225953</v>
-      </c>
-      <c r="F61">
-        <v>0.49963</v>
-      </c>
-      <c r="G61">
-        <v>-0.9979109712542467</v>
-      </c>
-      <c r="H61">
-        <v>0.04366557286781613</v>
+      <c r="E63">
+        <v>0.5906155179688426</v>
+      </c>
+      <c r="F63">
+        <v>0.49963</v>
+      </c>
+      <c r="G63">
+        <v>-0.9979109712542471</v>
+      </c>
+      <c r="H63">
+        <v>0.04366557286781612</v>
       </c>
     </row>
   </sheetData>

</xml_diff>